<commit_message>
Add backward tracing for animal origins and mortality explanation
Update Excel export with new sheets detailing animal origin tracing and a comprehensive explanation of mortality rates, alongside metadata title change.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 9581ce1c-c0df-4627-821a-5ac938c6c14e
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: a2d7bad5-50e9-44c3-a5d7-dcb53c312d5a
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2865e74a-6bcf-4df0-8524-8edc0c7c2777/9581ce1c-c0df-4627-821a-5ac938c6c14e/CCG2GRg
</commit_message>
<xml_diff>
--- a/exports/Bins_CaPisani_6-10_ciclo_penultimo-ultimo.xlsx
+++ b/exports/Bins_CaPisani_6-10_ciclo_penultimo-ultimo.xlsx
@@ -7,14 +7,16 @@
     <sheet sheetId="1" name="Sopravvivenza" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Penultimo ciclo" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Ultimo ciclo" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Vagliatura 129" state="visible" r:id="rId7"/>
+    <sheet sheetId="4" name="Origine (ritroso)" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Spiegazione mortalita" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Vagliatura 129" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="87">
   <si>
     <t>Sopravvivenza — Vagliatura #129 (16/06/2026)</t>
   </si>
@@ -104,6 +106,153 @@
   </si>
   <si>
     <t>misto 92+96</t>
+  </si>
+  <si>
+    <t>Ricostruzione a ritroso — da dove arrivano gli animali del PENULTIMO ciclo (bins 6-10)</t>
+  </si>
+  <si>
+    <t>Tipo origine</t>
+  </si>
+  <si>
+    <t>Provenienza</t>
+  </si>
+  <si>
+    <t>Animali sorgente</t>
+  </si>
+  <si>
+    <t>Perdita transito</t>
+  </si>
+  <si>
+    <t>Lotto seme</t>
+  </si>
+  <si>
+    <t>Trasferimento totale</t>
+  </si>
+  <si>
+    <t>01-03/06/2026</t>
+  </si>
+  <si>
+    <t>RACEWAY DF 5 - cesta #2</t>
+  </si>
+  <si>
+    <t>0%</t>
+  </si>
+  <si>
+    <t>92 - ROEM 0.35</t>
+  </si>
+  <si>
+    <t>Da vagliatura #111 (SOPRA)</t>
+  </si>
+  <si>
+    <t>Vagliatura #111 (pool 3 ceste)</t>
+  </si>
+  <si>
+    <t>(da pool)</t>
+  </si>
+  <si>
+    <t>misto 95/96/94</t>
+  </si>
+  <si>
+    <t>03-04/06/2026</t>
+  </si>
+  <si>
+    <t>BINS Delta Futuro - cesta #9</t>
+  </si>
+  <si>
+    <t>BINS Delta Futuro - cesta #10</t>
+  </si>
+  <si>
+    <t>TOTALE</t>
+  </si>
+  <si>
+    <t>Lotti seme di origine (acquisto/arrivo)</t>
+  </si>
+  <si>
+    <t>Fornitore</t>
+  </si>
+  <si>
+    <t>Arrivo</t>
+  </si>
+  <si>
+    <t>N. animali arrivati</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>ROEM 0.35</t>
+  </si>
+  <si>
+    <t>19/05/2026</t>
+  </si>
+  <si>
+    <t>Animali da ROEM in buone condizioni</t>
+  </si>
+  <si>
+    <t>Ecotapes Zeeland 0.3</t>
+  </si>
+  <si>
+    <t>21/05/2026</t>
+  </si>
+  <si>
+    <t>Animali da Zeeland belli</t>
+  </si>
+  <si>
+    <t>PERCHE LA MORTALITA E DEL 30,72% — SPIEGAZIONE</t>
+  </si>
+  <si>
+    <t>1) I conteggi di CARICO del penultimo ciclo (3-4 giugno) erano STIME riportate da:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Bin 6: trasferimento da RACEWAY DF 5 cesta #2 (270.338, lotto 92 ROEM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Bin 7-8: vagliatura #111 del 03/06 (2.829.545 ciascuno, lotto misto 95/96/94)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   - Bin 9-10: trasferimento da BINS Delta Futuro ceste #9 e #10 (2.100.555 / 2.100.554, lotto 92 ROEM)</t>
+  </si>
+  <si>
+    <t>2) Durante il penultimo ciclo (3-4/6 -&gt; 16/6, circa 12-13 giorni) NON e stata fatta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   nessuna misura intermedia: il conteggio e rimasto fermo alla stima di carico.</t>
+  </si>
+  <si>
+    <t>3) Alla vagliatura #129 (16/06) gli animali sono stati RICONTATI fisicamente a campione:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   risultato reale 7.018.874 contro i 10.130.537 stimati in carico.</t>
+  </si>
+  <si>
+    <t>4) La differenza di 3.111.663 (-30,72%) viene registrata tutta come MORTALITA al #129.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   Questa cifra unisce due cose:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   a) Mortalita reale del seme: sono animali piccolissimi (taglia TP-500, ~0,3-0,4 mg,</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      stadio larvale) con alta mortalita naturale, in piu manipolazioni e trasferimenti.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   b) Riconciliazione delle stime: i conteggi in ingresso erano essi stessi stime da</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      campionamento. Nota: la vagliatura #111 aveva chiuso addirittura in GUADAGNO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">      (9.988.803 -&gt; 10.123.251, +1,3%), segno che le stime a monte erano alte.</t>
+  </si>
+  <si>
+    <t>CONCLUSIONE: il 30,72% NON e necessariamente tutta morte avvenuta in 13 giorni, ma e la</t>
+  </si>
+  <si>
+    <t>somma tra mortalita reale del seme e la correzione delle stime al primo riconteggio reale.</t>
+  </si>
+  <si>
+    <t>Per avere un dato di mortalita piu preciso servirebbe una misura intermedia nel ciclo.</t>
   </si>
   <si>
     <t>ORIGINE (penultimo ciclo dei bins Ca Pisani 6-10)</t>
@@ -137,7 +286,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -161,6 +310,11 @@
       <b/>
       <color rgb="FF1F4E78"/>
       <sz val="13"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -188,18 +342,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -542,7 +697,7 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="42" customWidth="1"/>
+    <col min="1" max="1" width="44" customWidth="1"/>
     <col min="2" max="2" width="22" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1296,6 +1451,482 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I13"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="2" width="8" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="26" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="14" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <v>843</v>
+      </c>
+      <c r="C3" s="3">
+        <v>270338</v>
+      </c>
+      <c r="D3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F3" t="s">
+        <v>38</v>
+      </c>
+      <c r="G3" s="3">
+        <v>270338</v>
+      </c>
+      <c r="H3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>7</v>
+      </c>
+      <c r="B4">
+        <v>839</v>
+      </c>
+      <c r="C4" s="3">
+        <v>2829545</v>
+      </c>
+      <c r="D4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" t="s">
+        <v>42</v>
+      </c>
+      <c r="G4" s="3">
+        <v>2829545</v>
+      </c>
+      <c r="H4" t="s">
+        <v>43</v>
+      </c>
+      <c r="I4" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>8</v>
+      </c>
+      <c r="B5">
+        <v>840</v>
+      </c>
+      <c r="C5" s="3">
+        <v>2829545</v>
+      </c>
+      <c r="D5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>42</v>
+      </c>
+      <c r="G5" s="3">
+        <v>2829545</v>
+      </c>
+      <c r="H5" t="s">
+        <v>43</v>
+      </c>
+      <c r="I5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>9</v>
+      </c>
+      <c r="B6">
+        <v>844</v>
+      </c>
+      <c r="C6" s="3">
+        <v>2100555</v>
+      </c>
+      <c r="D6" t="s">
+        <v>36</v>
+      </c>
+      <c r="E6" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="3">
+        <v>2100555</v>
+      </c>
+      <c r="H6" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>10</v>
+      </c>
+      <c r="B7">
+        <v>845</v>
+      </c>
+      <c r="C7" s="3">
+        <v>2100554</v>
+      </c>
+      <c r="D7" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="3">
+        <v>2100554</v>
+      </c>
+      <c r="H7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="8">
+        <v>10130537</v>
+      </c>
+      <c r="D8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="G11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="I11" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>92</v>
+      </c>
+      <c r="B12" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="3">
+        <v>7835969</v>
+      </c>
+      <c r="E12" t="s">
+        <v>21</v>
+      </c>
+      <c r="F12" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" t="s">
+        <v>21</v>
+      </c>
+      <c r="H12" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>96</v>
+      </c>
+      <c r="B13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C13" t="s">
+        <v>58</v>
+      </c>
+      <c r="D13" s="3">
+        <v>5759000</v>
+      </c>
+      <c r="E13" t="s">
+        <v>21</v>
+      </c>
+      <c r="F13" t="s">
+        <v>59</v>
+      </c>
+      <c r="G13" t="s">
+        <v>21</v>
+      </c>
+      <c r="H13" t="s">
+        <v>21</v>
+      </c>
+      <c r="I13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A10:I10"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A24"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="100" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" s="9" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="9" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="9" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="9" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="9" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="9" t="s">
+        <v>78</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
@@ -1309,12 +1940,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>30</v>
+        <v>79</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>31</v>
+        <v>80</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>7</v>
@@ -1328,7 +1959,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="B3">
         <v>6</v>
@@ -1342,7 +1973,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="B4">
         <v>7</v>
@@ -1356,7 +1987,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="B5">
         <v>8</v>
@@ -1370,7 +2001,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="B6">
         <v>9</v>
@@ -1384,7 +2015,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="B7">
         <v>10</v>
@@ -1398,7 +2029,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>33</v>
+        <v>82</v>
       </c>
       <c r="B8" t="s">
         <v>21</v>
@@ -1412,12 +2043,12 @@
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
-        <v>34</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>31</v>
+        <v>80</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>7</v>
@@ -1440,7 +2071,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="B12">
         <v>6</v>
@@ -1463,7 +2094,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="B13">
         <v>7</v>
@@ -1486,7 +2117,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="B14">
         <v>8</v>
@@ -1509,7 +2140,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="B15">
         <v>9</v>
@@ -1532,7 +2163,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>32</v>
+        <v>81</v>
       </c>
       <c r="B16">
         <v>10</v>
@@ -1555,7 +2186,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="B17">
         <v>4</v>
@@ -1567,7 +2198,7 @@
         <v>138384</v>
       </c>
       <c r="E17" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="F17">
         <v>10</v>
@@ -1578,7 +2209,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="B18">
         <v>7</v>
@@ -1590,7 +2221,7 @@
         <v>138384</v>
       </c>
       <c r="E18" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="F18">
         <v>10</v>
@@ -1601,7 +2232,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="B19">
         <v>8</v>
@@ -1613,7 +2244,7 @@
         <v>138384</v>
       </c>
       <c r="E19" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="F19">
         <v>10</v>
@@ -1624,7 +2255,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="B20">
         <v>9</v>
@@ -1636,7 +2267,7 @@
         <v>138384</v>
       </c>
       <c r="E20" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="F20">
         <v>10</v>
@@ -1647,7 +2278,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="B21">
         <v>10</v>
@@ -1659,7 +2290,7 @@
         <v>138384</v>
       </c>
       <c r="E21" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="F21">
         <v>10</v>
@@ -1670,7 +2301,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>35</v>
+        <v>84</v>
       </c>
       <c r="B22">
         <v>11</v>
@@ -1682,7 +2313,7 @@
         <v>138384</v>
       </c>
       <c r="E22" t="s">
-        <v>36</v>
+        <v>85</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -1693,7 +2324,7 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>37</v>
+        <v>86</v>
       </c>
       <c r="B23" t="s">
         <v>21</v>

</xml_diff>

<commit_message>
Reconstruct bin genealogy to track animals back to original lots
Update Excel file with detailed genealogy of bins 6-10, tracing them back to their initial lot arrivals and suppliers.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 9581ce1c-c0df-4627-821a-5ac938c6c14e
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 855b6344-61a0-4cc4-8a5b-d498eb37b353
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/2865e74a-6bcf-4df0-8524-8edc0c7c2777/9581ce1c-c0df-4627-821a-5ac938c6c14e/CCG2GRg
</commit_message>
<xml_diff>
--- a/exports/Bins_CaPisani_6-10_ciclo_penultimo-ultimo.xlsx
+++ b/exports/Bins_CaPisani_6-10_ciclo_penultimo-ultimo.xlsx
@@ -7,16 +7,18 @@
     <sheet sheetId="1" name="Sopravvivenza" state="visible" r:id="rId4"/>
     <sheet sheetId="2" name="Penultimo ciclo" state="visible" r:id="rId5"/>
     <sheet sheetId="3" name="Ultimo ciclo" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="Origine (ritroso)" state="visible" r:id="rId7"/>
-    <sheet sheetId="5" name="Spiegazione mortalita" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Vagliatura 129" state="visible" r:id="rId9"/>
+    <sheet sheetId="4" name="Genealogia bins 6-10" state="visible" r:id="rId7"/>
+    <sheet sheetId="5" name="Composizione per lotto" state="visible" r:id="rId8"/>
+    <sheet sheetId="6" name="Lotti origine" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Spiegazione" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Vagliatura 129" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="363" uniqueCount="114">
   <si>
     <t>Sopravvivenza — Vagliatura #129 (16/06/2026)</t>
   </si>
@@ -87,7 +89,7 @@
     <t>TP-500</t>
   </si>
   <si>
-    <t>92</t>
+    <t>misto</t>
   </si>
   <si>
     <t>16/06/2026</t>
@@ -96,163 +98,244 @@
     <t>Chiusura (vagliatura #129)</t>
   </si>
   <si>
-    <t>96</t>
-  </si>
-  <si>
     <t>04/06/2026</t>
   </si>
   <si>
     <t>TP-1140</t>
   </si>
   <si>
-    <t>misto 92+96</t>
-  </si>
-  <si>
-    <t>Ricostruzione a ritroso — da dove arrivano gli animali del PENULTIMO ciclo (bins 6-10)</t>
-  </si>
-  <si>
-    <t>Tipo origine</t>
-  </si>
-  <si>
-    <t>Provenienza</t>
-  </si>
-  <si>
-    <t>Animali sorgente</t>
-  </si>
-  <si>
-    <t>Perdita transito</t>
-  </si>
-  <si>
-    <t>Lotto seme</t>
+    <t>GENEALOGIA — risalita fino al primo movimento del lotto</t>
+  </si>
+  <si>
+    <t>Passo</t>
+  </si>
+  <si>
+    <t>Evento / Movimento</t>
+  </si>
+  <si>
+    <t>Cesta / Destinazione</t>
+  </si>
+  <si>
+    <t>Lotti coinvolti</t>
+  </si>
+  <si>
+    <t>14/04 - 21/05</t>
+  </si>
+  <si>
+    <t>Arrivo lotti seme (primo movimento)</t>
+  </si>
+  <si>
+    <t>Magazzino</t>
+  </si>
+  <si>
+    <t>L75, L92, L93 (ROEM) + L97 (Zeeland 0.4)</t>
+  </si>
+  <si>
+    <t>01/06/2026</t>
+  </si>
+  <si>
+    <t>Vagliatura #107 (pool 4 ceste raceway)</t>
+  </si>
+  <si>
+    <t>-&gt; RACEWAY DF 5 #2 (ciclo 805)</t>
+  </si>
+  <si>
+    <t>92 64,7% / 93 5% / 97 13,5% / 75 16,8%</t>
   </si>
   <si>
     <t>Trasferimento totale</t>
   </si>
   <si>
-    <t>01-03/06/2026</t>
-  </si>
-  <si>
-    <t>RACEWAY DF 5 - cesta #2</t>
-  </si>
-  <si>
-    <t>0%</t>
-  </si>
-  <si>
-    <t>92 - ROEM 0.35</t>
-  </si>
-  <si>
-    <t>Da vagliatura #111 (SOPRA)</t>
+    <t>-&gt; BINS Ecotapes bin 6 (ciclo 843)</t>
+  </si>
+  <si>
+    <t>idem (misto)</t>
+  </si>
+  <si>
+    <t>Chiusura per vagliatura #129</t>
+  </si>
+  <si>
+    <t>bin 6</t>
+  </si>
+  <si>
+    <t>idem</t>
+  </si>
+  <si>
+    <t>-&gt; RACEWAY DF 5 #1 (ciclo 804)</t>
+  </si>
+  <si>
+    <t>Trasferimento 50% (split)</t>
+  </si>
+  <si>
+    <t>-&gt; BINS Delta Futuro #9 (ciclo 841)</t>
+  </si>
+  <si>
+    <t>-&gt; BINS Ecotapes bin 9 (ciclo 844)</t>
+  </si>
+  <si>
+    <t>bin 9</t>
+  </si>
+  <si>
+    <t>-&gt; BINS Delta Futuro #10 (ciclo 842)</t>
+  </si>
+  <si>
+    <t>-&gt; BINS Ecotapes bin 10 (ciclo 845)</t>
+  </si>
+  <si>
+    <t>bin 10</t>
+  </si>
+  <si>
+    <t>21/05/2026</t>
+  </si>
+  <si>
+    <t>L94, L95 (Zeeland 0.2) + L96 (Zeeland 0.3)</t>
+  </si>
+  <si>
+    <t>Prima attivazione da lotto</t>
+  </si>
+  <si>
+    <t>RACEWAY DF4#3 (L94), DF6#1 (L95), DF6#2 (L96)</t>
+  </si>
+  <si>
+    <t>3 ceste separate</t>
   </si>
   <si>
     <t>Vagliatura #111 (pool 3 ceste)</t>
   </si>
   <si>
-    <t>(da pool)</t>
-  </si>
-  <si>
-    <t>misto 95/96/94</t>
-  </si>
-  <si>
-    <t>03-04/06/2026</t>
-  </si>
-  <si>
-    <t>BINS Delta Futuro - cesta #9</t>
-  </si>
-  <si>
-    <t>BINS Delta Futuro - cesta #10</t>
+    <t>-&gt; BINS Ecotapes bin 7 (ciclo 839)</t>
+  </si>
+  <si>
+    <t>95 5,7% / 96 54,7% / 94 39,6%</t>
+  </si>
+  <si>
+    <t>bin 7</t>
+  </si>
+  <si>
+    <t>-&gt; BINS Ecotapes bin 8 (ciclo 840)</t>
+  </si>
+  <si>
+    <t>bin 8</t>
+  </si>
+  <si>
+    <t>Composizione REALE per lotto del penultimo ciclo (cestelli MISTI)</t>
+  </si>
+  <si>
+    <t>Fornitore</t>
+  </si>
+  <si>
+    <t>% nel cestello</t>
+  </si>
+  <si>
+    <t>ROEM 0.35</t>
+  </si>
+  <si>
+    <t>Zeeland 0.4</t>
+  </si>
+  <si>
+    <t>Zeeland 0.2</t>
+  </si>
+  <si>
+    <t>Zeeland 0.3</t>
+  </si>
+  <si>
+    <t>Totale per lotto (somma sui 5 bins origine)</t>
+  </si>
+  <si>
+    <t>% su origine</t>
   </si>
   <si>
     <t>TOTALE</t>
   </si>
   <si>
-    <t>Lotti seme di origine (acquisto/arrivo)</t>
-  </si>
-  <si>
-    <t>Fornitore</t>
+    <t>Lotti seme di origine — primo movimento</t>
   </si>
   <si>
     <t>Arrivo</t>
   </si>
   <si>
-    <t>N. animali arrivati</t>
-  </si>
-  <si>
-    <t>Note</t>
-  </si>
-  <si>
-    <t>ROEM 0.35</t>
+    <t>N. arrivati</t>
+  </si>
+  <si>
+    <t>Prima attivaz.</t>
+  </si>
+  <si>
+    <t>Prima cesta</t>
+  </si>
+  <si>
+    <t>14/04/2026</t>
+  </si>
+  <si>
+    <t>RACEWAY DF 1 #10</t>
   </si>
   <si>
     <t>19/05/2026</t>
   </si>
   <si>
-    <t>Animali da ROEM in buone condizioni</t>
+    <t>RACEWAY DF 4 #1</t>
+  </si>
+  <si>
+    <t>RACEWAY DF 3 #2</t>
+  </si>
+  <si>
+    <t>Ecotapes Zeeland 0.2</t>
+  </si>
+  <si>
+    <t>RACEWAY DF 4 #3</t>
+  </si>
+  <si>
+    <t>RACEWAY DF 6 #1</t>
   </si>
   <si>
     <t>Ecotapes Zeeland 0.3</t>
   </si>
   <si>
-    <t>21/05/2026</t>
-  </si>
-  <si>
-    <t>Animali da Zeeland belli</t>
-  </si>
-  <si>
-    <t>PERCHE LA MORTALITA E DEL 30,72% — SPIEGAZIONE</t>
-  </si>
-  <si>
-    <t>1) I conteggi di CARICO del penultimo ciclo (3-4 giugno) erano STIME riportate da:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - Bin 6: trasferimento da RACEWAY DF 5 cesta #2 (270.338, lotto 92 ROEM)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - Bin 7-8: vagliatura #111 del 03/06 (2.829.545 ciascuno, lotto misto 95/96/94)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   - Bin 9-10: trasferimento da BINS Delta Futuro ceste #9 e #10 (2.100.555 / 2.100.554, lotto 92 ROEM)</t>
-  </si>
-  <si>
-    <t>2) Durante il penultimo ciclo (3-4/6 -&gt; 16/6, circa 12-13 giorni) NON e stata fatta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   nessuna misura intermedia: il conteggio e rimasto fermo alla stima di carico.</t>
-  </si>
-  <si>
-    <t>3) Alla vagliatura #129 (16/06) gli animali sono stati RICONTATI fisicamente a campione:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   risultato reale 7.018.874 contro i 10.130.537 stimati in carico.</t>
-  </si>
-  <si>
-    <t>4) La differenza di 3.111.663 (-30,72%) viene registrata tutta come MORTALITA al #129.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   Questa cifra unisce due cose:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   a) Mortalita reale del seme: sono animali piccolissimi (taglia TP-500, ~0,3-0,4 mg,</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      stadio larvale) con alta mortalita naturale, in piu manipolazioni e trasferimenti.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">   b) Riconciliazione delle stime: i conteggi in ingresso erano essi stessi stime da</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      campionamento. Nota: la vagliatura #111 aveva chiuso addirittura in GUADAGNO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      (9.988.803 -&gt; 10.123.251, +1,3%), segno che le stime a monte erano alte.</t>
-  </si>
-  <si>
-    <t>CONCLUSIONE: il 30,72% NON e necessariamente tutta morte avvenuta in 13 giorni, ma e la</t>
-  </si>
-  <si>
-    <t>somma tra mortalita reale del seme e la correzione delle stime al primo riconteggio reale.</t>
-  </si>
-  <si>
-    <t>Per avere un dato di mortalita piu preciso servirebbe una misura intermedia nel ciclo.</t>
+    <t>RACEWAY DF 6 #2</t>
+  </si>
+  <si>
+    <t>Ecotapes Zeeland 0.4</t>
+  </si>
+  <si>
+    <t>RACEWAY DF 6 #3</t>
+  </si>
+  <si>
+    <t>DA DOVE ARRIVANO GLI ANIMALI (sintesi) — risalita ai lotti</t>
+  </si>
+  <si>
+    <t>Gli animali dei bins 6-10 vengono da DUE rami:</t>
+  </si>
+  <si>
+    <t>RAMO A -&gt; bins 6, 9, 10 (via Vagliatura #107 del 01/06):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Lotti 92, 93, 75 (ROEM 0.35) + 97 (Ecotapes Zeeland 0.4). Composizione ~ 92:64,7% 93:5% 97:13,5% 75:16,8%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Percorso: lotti -&gt; raceway -&gt; Vagliatura #107 -&gt; RACEWAY DF 5 (#1 e #2) -&gt; (DF5#1 split 50/50 in Delta Futuro #9 e #10) -&gt; bins 6/9/10.</t>
+  </si>
+  <si>
+    <t>RAMO B -&gt; bins 7, 8 (via Vagliatura #111 del 03/06):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Lotti 94, 95 (Ecotapes Zeeland 0.2) + 96 (Ecotapes Zeeland 0.3). Composizione ~ 95:5,7% 96:54,7% 94:39,6%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  Percorso: lotti -&gt; RACEWAY DF4#3 (L94), DF6#1 (L95), DF6#2 (L96) -&gt; Vagliatura #111 -&gt; bins 7/8.</t>
+  </si>
+  <si>
+    <t>PRIMO MOVIMENTO DEI LOTTI (arrivo in magazzino):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  L75 ROEM 0.35: 14/04/2026 (8.626.652)  |  L92 ROEM: 19/05 (7.835.969)  |  L93 ROEM: 19/05 (641.855)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  L94 Zeeland 0.2: 21/05 (4.410.000)  |  L95 Zeeland 0.2: 21/05 (1.050.000)  |  L96 Zeeland 0.3: 21/05 (5.759.000)  |  L97 Zeeland 0.4: 21/05 (1.644.651)</t>
+  </si>
+  <si>
+    <t>NOTA: ad ogni vagliatura i lotti vengono mescolati e ridistribuiti PRO-QUOTA. Per questo i numeri per singolo</t>
+  </si>
+  <si>
+    <t>lotto sono stime (non misure dirette) e la app segnala bassa confidenza sul lotto 92.</t>
   </si>
   <si>
     <t>ORIGINE (penultimo ciclo dei bins Ca Pisani 6-10)</t>
@@ -330,7 +413,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -338,11 +421,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF1F4E78"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -352,6 +444,7 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -771,7 +864,6 @@
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="8" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -923,7 +1015,7 @@
         <v>22</v>
       </c>
       <c r="L4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -999,7 +1091,7 @@
         <v>22</v>
       </c>
       <c r="L6" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -1048,7 +1140,7 @@
         <v>844</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" t="s">
         <v>20</v>
@@ -1124,7 +1216,7 @@
         <v>845</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D10" t="s">
         <v>20</v>
@@ -1212,7 +1304,6 @@
     <col min="8" max="8" width="15" customWidth="1"/>
     <col min="9" max="9" width="8" customWidth="1"/>
     <col min="10" max="10" width="12" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
@@ -1285,10 +1376,10 @@
         <v>0.054</v>
       </c>
       <c r="K2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L2" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1323,10 +1414,10 @@
         <v>0.054</v>
       </c>
       <c r="K3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L3" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1361,10 +1452,10 @@
         <v>0.054</v>
       </c>
       <c r="K4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L4" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -1399,10 +1490,10 @@
         <v>0.054</v>
       </c>
       <c r="K5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -1437,10 +1528,10 @@
         <v>0.054</v>
       </c>
       <c r="K6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="L6" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1451,340 +1542,561 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
-    <col min="4" max="4" width="26" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
-    <col min="6" max="6" width="32" customWidth="1"/>
-    <col min="7" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="7" customWidth="1"/>
+    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="4" max="4" width="34" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="G2" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="I2" s="5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>6</v>
       </c>
       <c r="B3">
-        <v>843</v>
-      </c>
-      <c r="C3" s="3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>2</v>
+      </c>
+      <c r="C4" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" t="s">
+        <v>38</v>
+      </c>
+      <c r="E4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="3">
         <v>270338</v>
       </c>
-      <c r="D3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F3" t="s">
-        <v>38</v>
-      </c>
-      <c r="G3" s="3">
-        <v>270338</v>
-      </c>
-      <c r="H3" t="s">
-        <v>39</v>
-      </c>
-      <c r="I3" t="s">
+      <c r="G4" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>7</v>
-      </c>
-      <c r="B4">
-        <v>839</v>
-      </c>
-      <c r="C4" s="3">
-        <v>2829545</v>
-      </c>
-      <c r="D4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" t="s">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
         <v>19</v>
-      </c>
-      <c r="F4" t="s">
-        <v>42</v>
-      </c>
-      <c r="G4" s="3">
-        <v>2829545</v>
-      </c>
-      <c r="H4" t="s">
-        <v>43</v>
-      </c>
-      <c r="I4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>8</v>
-      </c>
-      <c r="B5">
-        <v>840</v>
-      </c>
-      <c r="C5" s="3">
-        <v>2829545</v>
       </c>
       <c r="D5" t="s">
         <v>41</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F5" t="s">
         <v>42</v>
       </c>
-      <c r="G5" s="3">
-        <v>2829545</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="F5" s="3">
+        <v>270338</v>
+      </c>
+      <c r="G5" t="s">
         <v>43</v>
       </c>
-      <c r="I5" t="s">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>9</v>
-      </c>
-      <c r="B6">
-        <v>844</v>
-      </c>
-      <c r="C6" s="3">
-        <v>2100555</v>
-      </c>
-      <c r="D6" t="s">
-        <v>36</v>
       </c>
       <c r="E6" t="s">
         <v>45</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="3">
+        <v>270338</v>
+      </c>
+      <c r="G6" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="3">
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="7">
+        <v>9</v>
+      </c>
+      <c r="B7" s="7">
+        <v>1</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>9</v>
+      </c>
+      <c r="B8">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" t="s">
+        <v>47</v>
+      </c>
+      <c r="F8" s="3">
+        <v>4201109</v>
+      </c>
+      <c r="G8" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>9</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
+        <v>48</v>
+      </c>
+      <c r="E9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F9" s="3">
         <v>2100555</v>
       </c>
-      <c r="H6" t="s">
-        <v>39</v>
-      </c>
-      <c r="I6" t="s">
+      <c r="G9" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="3">
+        <v>2100555</v>
+      </c>
+      <c r="G10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>9</v>
+      </c>
+      <c r="B11">
+        <v>5</v>
+      </c>
+      <c r="C11" t="s">
+        <v>24</v>
+      </c>
+      <c r="D11" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" s="3">
+        <v>2100555</v>
+      </c>
+      <c r="G11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="7">
+        <v>10</v>
+      </c>
+      <c r="B12" s="7">
+        <v>1</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>10</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+      <c r="C13" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" t="s">
+        <v>38</v>
+      </c>
+      <c r="E13" t="s">
+        <v>47</v>
+      </c>
+      <c r="F13" s="3">
+        <v>4201109</v>
+      </c>
+      <c r="G13" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14">
         <v>10</v>
       </c>
-      <c r="B7">
-        <v>845</v>
-      </c>
-      <c r="C7" s="3">
+      <c r="B14">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" t="s">
+        <v>48</v>
+      </c>
+      <c r="E14" t="s">
+        <v>52</v>
+      </c>
+      <c r="F14" s="3">
         <v>2100554</v>
       </c>
-      <c r="D7" t="s">
-        <v>36</v>
-      </c>
-      <c r="E7" t="s">
-        <v>45</v>
-      </c>
-      <c r="F7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" s="3">
+      <c r="G14" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>10</v>
+      </c>
+      <c r="B15">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" t="s">
+        <v>53</v>
+      </c>
+      <c r="F15" s="3">
         <v>2100554</v>
       </c>
-      <c r="H7" t="s">
-        <v>39</v>
-      </c>
-      <c r="I7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="B8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8" s="8">
-        <v>10130537</v>
-      </c>
-      <c r="D8" t="s">
-        <v>21</v>
-      </c>
-      <c r="E8" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" t="s">
-        <v>21</v>
-      </c>
-      <c r="H8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I8" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>49</v>
-      </c>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I11" s="5" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <v>92</v>
-      </c>
-      <c r="B12" t="s">
+      <c r="G15" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>10</v>
+      </c>
+      <c r="B16">
+        <v>5</v>
+      </c>
+      <c r="C16" t="s">
+        <v>24</v>
+      </c>
+      <c r="D16" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" t="s">
         <v>54</v>
       </c>
-      <c r="C12" t="s">
+      <c r="F16" s="3">
+        <v>2100554</v>
+      </c>
+      <c r="G16" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="7">
+        <v>7</v>
+      </c>
+      <c r="B17" s="7">
+        <v>1</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D12" s="3">
-        <v>7835969</v>
-      </c>
-      <c r="E12" t="s">
-        <v>21</v>
-      </c>
-      <c r="F12" t="s">
+      <c r="D17" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F17" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="G12" t="s">
-        <v>21</v>
-      </c>
-      <c r="H12" t="s">
-        <v>21</v>
-      </c>
-      <c r="I12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13">
-        <v>96</v>
-      </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>7</v>
+      </c>
+      <c r="B18">
+        <v>2</v>
+      </c>
+      <c r="C18" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" t="s">
         <v>57</v>
       </c>
-      <c r="C13" t="s">
+      <c r="E18" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="3">
-        <v>5759000</v>
-      </c>
-      <c r="E13" t="s">
-        <v>21</v>
-      </c>
-      <c r="F13" t="s">
+      <c r="F18" t="s">
+        <v>21</v>
+      </c>
+      <c r="G18" t="s">
         <v>59</v>
       </c>
-      <c r="G13" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" t="s">
-        <v>21</v>
-      </c>
-      <c r="I13" t="s">
-        <v>21</v>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>7</v>
+      </c>
+      <c r="B19">
+        <v>3</v>
+      </c>
+      <c r="C19" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" t="s">
+        <v>60</v>
+      </c>
+      <c r="E19" t="s">
+        <v>61</v>
+      </c>
+      <c r="F19" s="3">
+        <v>2829545</v>
+      </c>
+      <c r="G19" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>7</v>
+      </c>
+      <c r="B20">
+        <v>4</v>
+      </c>
+      <c r="C20" t="s">
+        <v>24</v>
+      </c>
+      <c r="D20" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" t="s">
+        <v>63</v>
+      </c>
+      <c r="F20" s="3">
+        <v>2829545</v>
+      </c>
+      <c r="G20" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="7">
+        <v>8</v>
+      </c>
+      <c r="B21" s="7">
+        <v>1</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="F21" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>8</v>
+      </c>
+      <c r="B22">
+        <v>2</v>
+      </c>
+      <c r="C22" t="s">
+        <v>55</v>
+      </c>
+      <c r="D22" t="s">
+        <v>57</v>
+      </c>
+      <c r="E22" t="s">
+        <v>58</v>
+      </c>
+      <c r="F22" t="s">
+        <v>21</v>
+      </c>
+      <c r="G22" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>8</v>
+      </c>
+      <c r="B23">
+        <v>3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>19</v>
+      </c>
+      <c r="D23" t="s">
+        <v>60</v>
+      </c>
+      <c r="E23" t="s">
+        <v>64</v>
+      </c>
+      <c r="F23" s="3">
+        <v>2829545</v>
+      </c>
+      <c r="G23" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>8</v>
+      </c>
+      <c r="B24">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>24</v>
+      </c>
+      <c r="D24" t="s">
+        <v>44</v>
+      </c>
+      <c r="E24" t="s">
+        <v>65</v>
+      </c>
+      <c r="F24" s="3">
+        <v>2829545</v>
+      </c>
+      <c r="G24" t="s">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A10:I10"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1793,15 +2105,809 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A24"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="100" customWidth="1"/>
+    <col min="1" max="1" width="6" customWidth="1"/>
+    <col min="2" max="3" width="8" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="12" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>6</v>
+      </c>
+      <c r="B3">
+        <v>843</v>
+      </c>
+      <c r="C3">
+        <v>92</v>
+      </c>
+      <c r="D3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="3">
+        <v>175038</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0.6475</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>6</v>
+      </c>
+      <c r="B4">
+        <v>843</v>
+      </c>
+      <c r="C4">
+        <v>93</v>
+      </c>
+      <c r="D4" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" s="3">
+        <v>13440</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0.0497</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>6</v>
+      </c>
+      <c r="B5">
+        <v>843</v>
+      </c>
+      <c r="C5">
+        <v>97</v>
+      </c>
+      <c r="D5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E5" s="3">
+        <v>36496</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0.135</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>6</v>
+      </c>
+      <c r="B6">
+        <v>843</v>
+      </c>
+      <c r="C6">
+        <v>75</v>
+      </c>
+      <c r="D6" t="s">
+        <v>69</v>
+      </c>
+      <c r="E6" s="3">
+        <v>45364</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0.1678</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>839</v>
+      </c>
+      <c r="C7">
+        <v>95</v>
+      </c>
+      <c r="D7" t="s">
+        <v>71</v>
+      </c>
+      <c r="E7" s="3">
+        <v>160158</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0.0566</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>839</v>
+      </c>
+      <c r="C8">
+        <v>96</v>
+      </c>
+      <c r="D8" t="s">
+        <v>72</v>
+      </c>
+      <c r="E8" s="3">
+        <v>1548285</v>
+      </c>
+      <c r="F8" s="4">
+        <v>0.5472</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>7</v>
+      </c>
+      <c r="B9">
+        <v>839</v>
+      </c>
+      <c r="C9">
+        <v>94</v>
+      </c>
+      <c r="D9" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1121102</v>
+      </c>
+      <c r="F9" s="4">
+        <v>0.3962</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>8</v>
+      </c>
+      <c r="B10">
+        <v>840</v>
+      </c>
+      <c r="C10">
+        <v>95</v>
+      </c>
+      <c r="D10" t="s">
+        <v>71</v>
+      </c>
+      <c r="E10" s="3">
+        <v>160158</v>
+      </c>
+      <c r="F10" s="4">
+        <v>0.0566</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>8</v>
+      </c>
+      <c r="B11">
+        <v>840</v>
+      </c>
+      <c r="C11">
+        <v>96</v>
+      </c>
+      <c r="D11" t="s">
+        <v>72</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1548285</v>
+      </c>
+      <c r="F11" s="4">
+        <v>0.5472</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>8</v>
+      </c>
+      <c r="B12">
+        <v>840</v>
+      </c>
+      <c r="C12">
+        <v>94</v>
+      </c>
+      <c r="D12" t="s">
+        <v>71</v>
+      </c>
+      <c r="E12" s="3">
+        <v>1121102</v>
+      </c>
+      <c r="F12" s="4">
+        <v>0.3962</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13">
+        <v>9</v>
+      </c>
+      <c r="B13">
+        <v>844</v>
+      </c>
+      <c r="C13">
+        <v>92</v>
+      </c>
+      <c r="D13" t="s">
+        <v>69</v>
+      </c>
+      <c r="E13" s="3">
+        <v>1360065</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0.6475</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>9</v>
+      </c>
+      <c r="B14">
+        <v>844</v>
+      </c>
+      <c r="C14">
+        <v>93</v>
+      </c>
+      <c r="D14" t="s">
+        <v>69</v>
+      </c>
+      <c r="E14" s="3">
+        <v>104433</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0.0497</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15">
+        <v>9</v>
+      </c>
+      <c r="B15">
+        <v>844</v>
+      </c>
+      <c r="C15">
+        <v>97</v>
+      </c>
+      <c r="D15" t="s">
+        <v>70</v>
+      </c>
+      <c r="E15" s="3">
+        <v>283575</v>
+      </c>
+      <c r="F15" s="4">
+        <v>0.135</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16">
+        <v>9</v>
+      </c>
+      <c r="B16">
+        <v>844</v>
+      </c>
+      <c r="C16">
+        <v>75</v>
+      </c>
+      <c r="D16" t="s">
+        <v>69</v>
+      </c>
+      <c r="E16" s="3">
+        <v>352482</v>
+      </c>
+      <c r="F16" s="4">
+        <v>0.1678</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>10</v>
+      </c>
+      <c r="B17">
+        <v>845</v>
+      </c>
+      <c r="C17">
+        <v>92</v>
+      </c>
+      <c r="D17" t="s">
+        <v>69</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1360064</v>
+      </c>
+      <c r="F17" s="4">
+        <v>0.6475</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>10</v>
+      </c>
+      <c r="B18">
+        <v>845</v>
+      </c>
+      <c r="C18">
+        <v>93</v>
+      </c>
+      <c r="D18" t="s">
+        <v>69</v>
+      </c>
+      <c r="E18" s="3">
+        <v>104434</v>
+      </c>
+      <c r="F18" s="4">
+        <v>0.0497</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>10</v>
+      </c>
+      <c r="B19">
+        <v>845</v>
+      </c>
+      <c r="C19">
+        <v>97</v>
+      </c>
+      <c r="D19" t="s">
+        <v>70</v>
+      </c>
+      <c r="E19" s="3">
+        <v>283574</v>
+      </c>
+      <c r="F19" s="4">
+        <v>0.135</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>10</v>
+      </c>
+      <c r="B20">
+        <v>845</v>
+      </c>
+      <c r="C20">
+        <v>75</v>
+      </c>
+      <c r="D20" t="s">
+        <v>69</v>
+      </c>
+      <c r="E20" s="3">
+        <v>352482</v>
+      </c>
+      <c r="F20" s="4">
+        <v>0.1678</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>21</v>
+      </c>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24">
+        <v>96</v>
+      </c>
+      <c r="D24" t="s">
+        <v>72</v>
+      </c>
+      <c r="E24" s="3">
+        <v>3096570</v>
+      </c>
+      <c r="F24" s="4">
+        <v>0.3056669157814635</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" t="s">
+        <v>21</v>
+      </c>
+      <c r="C25">
+        <v>92</v>
+      </c>
+      <c r="D25" t="s">
+        <v>69</v>
+      </c>
+      <c r="E25" s="3">
+        <v>2895167</v>
+      </c>
+      <c r="F25" s="4">
+        <v>0.28578613354849797</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26">
+        <v>94</v>
+      </c>
+      <c r="D26" t="s">
+        <v>71</v>
+      </c>
+      <c r="E26" s="3">
+        <v>2242204</v>
+      </c>
+      <c r="F26" s="4">
+        <v>0.22133120879969148</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27" t="s">
+        <v>21</v>
+      </c>
+      <c r="C27">
+        <v>75</v>
+      </c>
+      <c r="D27" t="s">
+        <v>69</v>
+      </c>
+      <c r="E27" s="3">
+        <v>750328</v>
+      </c>
+      <c r="F27" s="4">
+        <v>0.07406596511122757</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" t="s">
+        <v>21</v>
+      </c>
+      <c r="C28">
+        <v>97</v>
+      </c>
+      <c r="D28" t="s">
+        <v>70</v>
+      </c>
+      <c r="E28" s="3">
+        <v>603645</v>
+      </c>
+      <c r="F28" s="4">
+        <v>0.059586673440904465</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>21</v>
+      </c>
+      <c r="B29" t="s">
+        <v>21</v>
+      </c>
+      <c r="C29">
+        <v>95</v>
+      </c>
+      <c r="D29" t="s">
+        <v>71</v>
+      </c>
+      <c r="E29" s="3">
+        <v>320316</v>
+      </c>
+      <c r="F29" s="4">
+        <v>0.03161885692732774</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>21</v>
+      </c>
+      <c r="B30" t="s">
+        <v>21</v>
+      </c>
+      <c r="C30">
+        <v>93</v>
+      </c>
+      <c r="D30" t="s">
+        <v>69</v>
+      </c>
+      <c r="E30" s="3">
+        <v>222307</v>
+      </c>
+      <c r="F30" s="4">
+        <v>0.021944246390887275</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>21</v>
+      </c>
+      <c r="B31" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D31" t="s">
+        <v>21</v>
+      </c>
+      <c r="E31" s="9">
+        <v>10130537</v>
+      </c>
+      <c r="F31" s="4">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A22:F22"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>75</v>
+      </c>
+      <c r="B3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D3" s="3">
+        <v>8626652</v>
+      </c>
+      <c r="E3" t="s">
+        <v>81</v>
+      </c>
+      <c r="F3" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>92</v>
+      </c>
+      <c r="B4" t="s">
+        <v>69</v>
+      </c>
+      <c r="C4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D4" s="3">
+        <v>7835969</v>
+      </c>
+      <c r="E4" t="s">
+        <v>83</v>
+      </c>
+      <c r="F4" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>93</v>
+      </c>
+      <c r="B5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D5" s="3">
+        <v>641855</v>
+      </c>
+      <c r="E5" t="s">
+        <v>83</v>
+      </c>
+      <c r="F5" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>94</v>
+      </c>
+      <c r="B6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="3">
+        <v>4410000</v>
+      </c>
+      <c r="E6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>95</v>
+      </c>
+      <c r="B7" t="s">
+        <v>86</v>
+      </c>
+      <c r="C7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1050000</v>
+      </c>
+      <c r="E7" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>96</v>
+      </c>
+      <c r="B8" t="s">
+        <v>89</v>
+      </c>
+      <c r="C8" t="s">
+        <v>55</v>
+      </c>
+      <c r="D8" s="3">
+        <v>5759000</v>
+      </c>
+      <c r="E8" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>97</v>
+      </c>
+      <c r="B9" t="s">
+        <v>91</v>
+      </c>
+      <c r="C9" t="s">
+        <v>55</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1644651</v>
+      </c>
+      <c r="E9" t="s">
+        <v>55</v>
+      </c>
+      <c r="F9" t="s">
+        <v>92</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A18"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="104" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>60</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -1810,113 +2916,83 @@
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" s="9" t="s">
-        <v>61</v>
+      <c r="A3" s="10" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>63</v>
+      <c r="A5" s="10" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>64</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" s="9" t="s">
-        <v>65</v>
+      <c r="A8" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>66</v>
+      <c r="A9" s="10" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" s="9" t="s">
-        <v>67</v>
+      <c r="A11" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>21</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>21</v>
+      <c r="A13" s="10" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" s="9" t="s">
-        <v>69</v>
+      <c r="A14" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>70</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>71</v>
+        <v>21</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>72</v>
+      <c r="A17" s="10" t="s">
+        <v>104</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" s="9" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" s="9" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" s="9" t="s">
-        <v>78</v>
+      <c r="A18" s="10" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -1925,7 +3001,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1939,13 +3015,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
-        <v>79</v>
+      <c r="A1" s="8" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>80</v>
+        <v>107</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>7</v>
@@ -1959,7 +3035,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="B3">
         <v>6</v>
@@ -1973,7 +3049,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="B4">
         <v>7</v>
@@ -1987,7 +3063,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="B5">
         <v>8</v>
@@ -2001,7 +3077,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="B6">
         <v>9</v>
@@ -2015,7 +3091,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="B7">
         <v>10</v>
@@ -2029,12 +3105,12 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>82</v>
+        <v>109</v>
       </c>
       <c r="B8" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="8">
+      <c r="C8" s="9">
         <v>10130537</v>
       </c>
       <c r="D8" t="s">
@@ -2042,13 +3118,13 @@
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7" t="s">
-        <v>83</v>
+      <c r="A10" s="8" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>80</v>
+        <v>107</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>7</v>
@@ -2071,7 +3147,7 @@
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="B12">
         <v>6</v>
@@ -2083,7 +3159,7 @@
         <v>336554</v>
       </c>
       <c r="E12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F12">
         <v>12</v>
@@ -2094,7 +3170,7 @@
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="B13">
         <v>7</v>
@@ -2106,7 +3182,7 @@
         <v>336554</v>
       </c>
       <c r="E13" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F13">
         <v>12</v>
@@ -2117,7 +3193,7 @@
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="B14">
         <v>8</v>
@@ -2129,7 +3205,7 @@
         <v>336554</v>
       </c>
       <c r="E14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F14">
         <v>12</v>
@@ -2140,7 +3216,7 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="B15">
         <v>9</v>
@@ -2152,7 +3228,7 @@
         <v>336554</v>
       </c>
       <c r="E15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F15">
         <v>12</v>
@@ -2163,7 +3239,7 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>81</v>
+        <v>108</v>
       </c>
       <c r="B16">
         <v>10</v>
@@ -2175,7 +3251,7 @@
         <v>336554</v>
       </c>
       <c r="E16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F16">
         <v>12</v>
@@ -2186,7 +3262,7 @@
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="B17">
         <v>4</v>
@@ -2198,7 +3274,7 @@
         <v>138384</v>
       </c>
       <c r="E17" t="s">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="F17">
         <v>10</v>
@@ -2209,7 +3285,7 @@
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="B18">
         <v>7</v>
@@ -2221,7 +3297,7 @@
         <v>138384</v>
       </c>
       <c r="E18" t="s">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="F18">
         <v>10</v>
@@ -2232,7 +3308,7 @@
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="B19">
         <v>8</v>
@@ -2244,7 +3320,7 @@
         <v>138384</v>
       </c>
       <c r="E19" t="s">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="F19">
         <v>10</v>
@@ -2255,7 +3331,7 @@
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="B20">
         <v>9</v>
@@ -2267,7 +3343,7 @@
         <v>138384</v>
       </c>
       <c r="E20" t="s">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="F20">
         <v>10</v>
@@ -2278,7 +3354,7 @@
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="B21">
         <v>10</v>
@@ -2290,7 +3366,7 @@
         <v>138384</v>
       </c>
       <c r="E21" t="s">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="F21">
         <v>10</v>
@@ -2301,7 +3377,7 @@
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>84</v>
+        <v>111</v>
       </c>
       <c r="B22">
         <v>11</v>
@@ -2313,7 +3389,7 @@
         <v>138384</v>
       </c>
       <c r="E22" t="s">
-        <v>85</v>
+        <v>112</v>
       </c>
       <c r="F22">
         <v>10</v>
@@ -2324,12 +3400,12 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>86</v>
+        <v>113</v>
       </c>
       <c r="B23" t="s">
         <v>21</v>
       </c>
-      <c r="C23" s="8">
+      <c r="C23" s="9">
         <v>7018874</v>
       </c>
       <c r="D23" t="s">

</xml_diff>